<commit_message>
update data for stat signif
</commit_message>
<xml_diff>
--- a/data/PL_D21_Spleen_CFU_data.xlsx
+++ b/data/PL_D21_Spleen_CFU_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11108"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henaolab/Documents/R/bactcountr_shiny/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0200C391-C9D3-8F4E-8330-AEED2E4C1867}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A13764-DD80-2349-AF33-319582272BA4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24900" yWindow="1960" windowWidth="19840" windowHeight="22380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>group</t>
   </si>
   <si>
-    <t>mouse</t>
-  </si>
-  <si>
     <t>dilution_0</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>TNTC</t>
+  </si>
+  <si>
+    <t>replicate</t>
   </si>
 </sst>
 </file>
@@ -525,19 +525,19 @@
         <v>13</v>
       </c>
       <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>17</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -545,7 +545,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2">
         <v>48</v>
@@ -565,13 +565,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2">
         <v>58</v>
@@ -585,10 +585,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2">
         <v>81</v>
@@ -605,10 +605,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
@@ -625,7 +625,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2">
         <v>14</v>
@@ -645,10 +645,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2">
         <v>32</v>
@@ -665,10 +665,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2">
         <v>21</v>
@@ -685,13 +685,13 @@
         <v>3</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="2">
         <v>29</v>
@@ -705,10 +705,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="2">
         <v>83</v>
@@ -725,10 +725,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" s="2">
         <v>36</v>
@@ -745,10 +745,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" s="2">
         <v>31</v>
@@ -765,10 +765,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2">
         <v>38</v>
@@ -785,7 +785,7 @@
         <v>5</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2">
         <v>10</v>
@@ -805,7 +805,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2">
         <v>31</v>
@@ -825,10 +825,10 @@
         <v>5</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" s="2">
         <v>54</v>
@@ -845,10 +845,10 @@
         <v>6</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" s="2">
         <v>50</v>
@@ -865,13 +865,13 @@
         <v>6</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E18" s="2">
         <v>22</v>
@@ -885,16 +885,16 @@
         <v>6</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F19" s="2">
         <v>177</v>
@@ -905,7 +905,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="2">
         <v>32</v>
@@ -925,7 +925,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2">
         <v>40</v>
@@ -945,7 +945,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2">
         <v>68</v>
@@ -965,10 +965,10 @@
         <v>8</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" s="2">
         <v>24</v>
@@ -977,7 +977,7 @@
         <v>7</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -985,7 +985,7 @@
         <v>8</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" s="2">
         <v>20</v>
@@ -1005,10 +1005,10 @@
         <v>8</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D25" s="2">
         <v>69</v>
@@ -1025,7 +1025,7 @@
         <v>9</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -1045,7 +1045,7 @@
         <v>9</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
@@ -1065,7 +1065,7 @@
         <v>9</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C28" s="2">
         <v>40</v>
@@ -1085,7 +1085,7 @@
         <v>10</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C29" s="2">
         <v>0</v>
@@ -1105,10 +1105,10 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D30" s="2">
         <v>69</v>
@@ -1125,13 +1125,13 @@
         <v>10</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E31" s="2">
         <v>34</v>

</xml_diff>